<commit_message>
feat(web-platform): update cms project audit, hub brds, roadmaps and reports
</commit_message>
<xml_diff>
--- a/05_HUBS/vehicle-hub-roadmap.xlsx
+++ b/05_HUBS/vehicle-hub-roadmap.xlsx
@@ -10,10 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Sizing &amp; Opportunities" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs &amp; Target Metrics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI &amp; Resource Allocation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilities &amp; Formula Specs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Tracking Spec" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Structure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs &amp; Target Metrics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI &amp; Resource Allocation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilities &amp; Formula Specs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Tracking Spec" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,7 +179,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -214,8 +215,43 @@
         <fgColor rgb="000B5394"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B6D7A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004C1130"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -321,11 +357,32 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -510,6 +567,62 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1293,14 +1406,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1357,559 +1470,283 @@
       </c>
     </row>
     <row r="4" ht="68" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Phase 1: Build-Up (Nền Tảng Tiện Ích Lõi - 25/08 đến 25/09/2026)</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Master Hub Gateway</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="A4" s="98" t="inlineStr">
+        <is>
+          <t>Phase 1.0: Master Hub Launch (Cuối Tháng 8/2026)</t>
+        </is>
+      </c>
+      <c r="B4" s="99" t="inlineStr">
+        <is>
+          <t>Master Hub</t>
+        </is>
+      </c>
+      <c r="C4" s="100" t="inlineStr">
         <is>
           <t>Trang Chủ Master Hub (/tien-ich-giao-thong)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Dựng mặt tiền trung tâm hợp nhất toàn bộ dịch vụ xe trên Open Web
-2. Tích hợp Widget 3-in-1 trước khi lăn bánh (Tra cứu phạt nguội, Giá xăng, ePass/BOT)
-3. Khối Value Exchange Block (Thẻ Xe Số MoMo - 1 chiếc xe, 1 tài khoản)
-4. Thiết lập Header Menu chuẩn 6 cụm &amp; Dynamic QR Code (Desktop) / Onelink (Mobile)</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Giữa Tháng (15/09) &amp; Go-live (25/09)</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform (Chủ trì A/R) | InsurTech &amp; VTTI (Onelink)</t>
+      <c r="D4" s="100" t="inlineStr">
+        <is>
+          <t>Lên sóng mặt tiền trung tâm hệ sinh thái tiện ích giao thông (Hero Widget, Navigation).</t>
+        </is>
+      </c>
+      <c r="E4" s="99" t="inlineStr">
+        <is>
+          <t>Cuối Tháng 8/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="68" customHeight="1">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Daily Fuel &amp; Utilities</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Bảng Giá Xăng Dầu (/gia-xang)</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>1. Cập nhật bảng giá xăng RON 95, E5, Diesel realtime lúc 15:00 thứ Năm hàng tuần theo Bộ Công Thương
-2. Biểu đồ biến động giá xăng 6 tháng gần nhất &amp; công cụ tính tiền đầy bình xăng
-3. Tối ưu SEO cụm 'giá xăng hôm nay' (10.52M search demand)
-Vai trò: Traffic Magnet giữ chân người dùng hàng ngày</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Check-in Đầu Sprint &amp; Go-live (25/09)</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform (Code Web) | Content Team (Bài Viết)</t>
+      <c r="A5" s="93" t="inlineStr">
+        <is>
+          <t>Phase 1.1: Traffic Magnets (Tuần 1-2 Tháng 9/2026)</t>
+        </is>
+      </c>
+      <c r="B5" s="83" t="inlineStr">
+        <is>
+          <t>Magnet + Transaction</t>
+        </is>
+      </c>
+      <c r="C5" s="84" t="inlineStr">
+        <is>
+          <t>Mở rộng Phạt Nguội &amp; Location Page (/phat-nguoi, /phat-nguoi/[tinh])</t>
+        </is>
+      </c>
+      <c r="D5" s="84" t="inlineStr">
+        <is>
+          <t>Mở rộng trang Phạt nguội theo tỉnh/thành. Đẩy mạnh traffic dẫn về luồng Nộp Phạt In-App.</t>
+        </is>
+      </c>
+      <c r="E5" s="83" t="inlineStr">
+        <is>
+          <t>Tuần 1-2 (Tháng 9)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="68" customHeight="1">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Daily Fuel &amp; Utilities</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Bản Đồ Cây Xăng Gần Nhất (/cay-xang)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>1. Bản đồ định vị cây xăng Petrolimex/PVOil/Comeco chấp nhận quét mã MoMo theo GPS
-2. Tiếp nhận dữ liệu cây xăng qua Google Sheet đồng bộ tự động vào CDN (Batch Sync)
-3. Nút 1-click 'Chỉ đường Google Maps' &amp; nhận Voucher xăng MoMo
-Vai trò: O2O Payment Bridge &amp; GPS Local Utility (550K search)</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Nhận Data (11/09) &amp; Go-live (25/09)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform (Map UI) | VTTI (Cung Cấp Data)</t>
+      <c r="A6" s="86" t="n"/>
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t>Location (High Volume)</t>
+        </is>
+      </c>
+      <c r="C6" s="84" t="inlineStr">
+        <is>
+          <t>Giá Xăng &amp; Cây Xăng (/gia-xang, /cay-xang)</t>
+        </is>
+      </c>
+      <c r="D6" s="84" t="inlineStr">
+        <is>
+          <t>Cập nhật giá xăng realtime và bản đồ định vị cây xăng để hứng traffic cực lớn (&gt;10M).</t>
+        </is>
+      </c>
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t>Tuần 1-2 (Tháng 9)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="68" customHeight="1">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Daily Fuel &amp; Utilities</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Trạm Sạc Xe Điện EV (/tram-sac &amp; /tram-sac/vinfast)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>1. Bản đồ trạm sạc VinFast, V-Green toàn quốc theo GPS thời gian thực
-2. Bộ lọc trụ sạc siêu nhanh DC/AC theo công suất và loại xe (Ô tô điện / Xe máy điện)
-3. Tối ưu SEO cụm 'trạm sạc vinfast gần nhất' (1.24M search demand)
-Vai trò: Tiếp cận tệp khách hàng xe điện hiện đại</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Check-in Nhận Data (11/09) &amp; Go-live (25/09)</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform (Map UI) | VTTI (Data Trạm Sạc)</t>
+      <c r="A7" s="95" t="inlineStr">
+        <is>
+          <t>Phase 1.2: Maps Expansion &amp; Content (Tuần 3-4 Tháng 9/2026)</t>
+        </is>
+      </c>
+      <c r="B7" s="96" t="inlineStr">
+        <is>
+          <t>Location &amp; Maps</t>
+        </is>
+      </c>
+      <c r="C7" s="97" t="inlineStr">
+        <is>
+          <t>Bản đồ Trạm sạc, Bãi đỗ &amp; Rửa xe (/tram-sac, /bai-do-xe, /bao-duong)</t>
+        </is>
+      </c>
+      <c r="D7" s="97" t="inlineStr">
+        <is>
+          <t>Xây dựng bản đồ định vị Garage/Rửa xe, Trạm sạc EV, Bãi đỗ xe.</t>
+        </is>
+      </c>
+      <c r="E7" s="96" t="inlineStr">
+        <is>
+          <t>Tuần 3-4 (Tháng 9)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="68" customHeight="1">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Care</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Bản Đồ Garage &amp; Vá Lốp (/tim-garage)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>1. Định vị tiệm sửa xe, garage bảo dưỡng, vá lốp khẩn cấp gần nhất theo vị trí người dùng
-2. Tích hợp bảng giá dịch vụ tham khảo &amp; hotline gọi trực tiếp
-3. Tiếp nhận danh bạ garage qua Google Sheet Algify
-Vai trò: Tiện ích hỗ trợ khẩn cấp &amp; O2O Garage Network (934K search)</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Nhận Data (11/09) &amp; Go-live (25/09)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform (Map UI) | VTTI (Data Garage)</t>
+      <c r="A8" s="85" t="n"/>
+      <c r="B8" s="96" t="inlineStr">
+        <is>
+          <t>Content &amp; SEO</t>
+        </is>
+      </c>
+      <c r="C8" s="97" t="inlineStr">
+        <is>
+          <t>Blog &amp; Content Production (/tra-cuu-muc-phat, /bien-bao-giao-thong)</t>
+        </is>
+      </c>
+      <c r="D8" s="97" t="inlineStr">
+        <is>
+          <t>Sản xuất nội dung cẩm nang, tra cứu mức phạt NĐ 100/123, biển báo, kinh nghiệm.</t>
+        </is>
+      </c>
+      <c r="E8" s="96" t="inlineStr">
+        <is>
+          <t>Tuần 3-4 (Tháng 9)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="68" customHeight="1">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Mobility &amp; Toll</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Biểu Phí BOT &amp; Nạp ePass (/tram-thu-phi &amp; /epass)</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>1. Tra cứu biểu phí các trạm thu phí BOT toàn quốc &amp; hướng dẫn liên kết nạp tiền ePass/VETC
-2. Hướng dẫn kích hoạt tính năng Auto-Topup tự động bù tiền khi qua trạm BOT
-3. Nút W2A CTA dẫn mở App MoMo nạp tiền thu phí không dừng tức thì
-Vai trò: Flagship Utility (95K search)</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Check-in ePass API (15/09) &amp; Go-live (25/09)</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform (Xây Web) | VTTI (API ePass)</t>
+      <c r="A9" s="86" t="n"/>
+      <c r="B9" s="96" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="C9" s="97" t="inlineStr">
+        <is>
+          <t>Tra Cứu Hạn Đăng Kiểm (/dang-kiem)</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>Xây dựng trang tra cứu hạn đăng kiểm &amp; đặt lịch kiểm định.</t>
+        </is>
+      </c>
+      <c r="E9" s="96" t="inlineStr">
+        <is>
+          <t>Tuần 3-4 (Tháng 9)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="68" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Tối Ưu Hiệu Năng &amp; Bản Đồ Địa Lý</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Tối Ưu Hiệu Năng Tải Trang &amp; Khả Năng Tiếp Cận</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>1. Tối ưu hóa On-Page SEO, cấu trúc đường dẫn và tốc độ tải trang trên nền tảng MoSpark CMS
-2. Nhúng Schema dữ liệu có cấu trúc JSON-LD chuẩn Google (LocalBusiness, GeoCoordinates, FAQPage)
-3. Tối ưu Local GEO và định vị GPS cho bản đồ Cây xăng, Trạm sạc EV, Garage Top 5 Tỉnh/Thành
-Vai trò: Đảm bảo thứ hạng tìm kiếm và khả năng hiển thị Rich Snippets trước Go-live 25/09</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Nghiệm thu On-Page (28/08)</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform (Dev Lead &amp; Growth)</t>
+      <c r="A10" s="94" t="inlineStr">
+        <is>
+          <t>Phase 2: Giao dịch, Tài chính &amp; Khẩn Cấp (Tháng 10/2026)</t>
+        </is>
+      </c>
+      <c r="B10" s="87" t="inlineStr">
+        <is>
+          <t>Transaction (Mở rộng)</t>
+        </is>
+      </c>
+      <c r="C10" s="88" t="inlineStr">
+        <is>
+          <t>Thu Phí BOT (/phi-khong-dung, /tram-thu-phi)</t>
+        </is>
+      </c>
+      <c r="D10" s="88" t="inlineStr">
+        <is>
+          <t>Phát triển &amp; mở rộng luồng nạp tiền thu phí không dừng ePass/VETC đã build.</t>
+        </is>
+      </c>
+      <c r="E10" s="87" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
         </is>
       </c>
     </row>
     <row r="11" ht="68" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Phase 2: Expansion (Mở Rộng Tiện Ích &amp; Pháp Lý - Tháng 10/2026)</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Legal &amp; Compliance</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Phễu Phạt Nguội &amp; Cẩm Nang Luật (/phat-nguoi/*)</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>1. Tối ưu trang Phạt Nguội (/phat-nguoi, /ha-noi, /nop-qua-momo, /giai-dap, /tra-cuu-luat)
-2. Phân nhánh trả kết quả thông minh: Có lỗi (Nộp phạt In-App + Trích dẫn luật NĐ 100/123) / Không lỗi (Tặng voucher Bảo hiểm TNDS)
-3. Nút W2A 'Bật thông báo phạt nguội tự động thứ Hai hàng tuần'
-Vai trò: Đầu phễu hút khách lớn nhất (6.1M traffic) &amp; thu thập biển số xe</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Check-in Giữa Tháng 10 &amp; Review Cuối Tháng 10</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech Cell | Content Team</t>
+      <c r="A11" s="85" t="n"/>
+      <c r="B11" s="87" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="C11" s="88" t="inlineStr">
+        <is>
+          <t>Cứu Hộ Ô Tô (/cuu-ho)</t>
+        </is>
+      </c>
+      <c r="D11" s="88" t="inlineStr">
+        <is>
+          <t>Danh bạ bản đồ gọi cứu hộ ô tô khẩn cấp 24/7.</t>
+        </is>
+      </c>
+      <c r="E11" s="87" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
         </is>
       </c>
     </row>
     <row r="12" ht="68" customHeight="1">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Pre-Purchase &amp; Evaluation</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Bộ Công Cụ Tính Toán Giá Lăn Bánh &amp; Chi Phí (/lan-banh, /chi-phi-nuoi-xe, /so-sanh-xe)</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>1. Công cụ tính giá lăn bánh ô tô theo 63 tỉnh thành (thuế trước bạ, biển số, phí đường bộ)
-2. Máy tính chi phí nuôi xe hàng tháng (xăng, gửi xe, bảo dưỡng, bảo hiểm)
-3. Đặt lên bàn cân so sánh 2-3 mẫu xe
-Vai trò: Hứng traffic nhóm Mua xe &amp; dẫn luồng mua Bảo hiểm / Vay mua xe</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Giữa Tháng 10 &amp; Review Cuối Tháng 10</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech Cell</t>
+      <c r="A12" s="85" t="n"/>
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>Monetize</t>
+        </is>
+      </c>
+      <c r="C12" s="88" t="inlineStr">
+        <is>
+          <t>Bảo Hiểm Phương Tiện (/bao-hiem-o-to, /bao-hiem-xe-may)</t>
+        </is>
+      </c>
+      <c r="D12" s="88" t="inlineStr">
+        <is>
+          <t>Luồng cross-sell bảo hiểm, prefill thông tin xe.</t>
+        </is>
+      </c>
+      <c r="E12" s="87" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
         </is>
       </c>
     </row>
     <row r="13" ht="68" customHeight="1">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Compliance &amp; Licensing</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Đăng Kiểm Xe &amp; Tra Cứu 12 Điểm GPLX (/dang-kiem, /diem-gplx, /sang-ten-xe, /bien-so-xe)</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>1. Tra cứu chu kỳ kiểm định, hạn đăng kiểm &amp; đặt lịch kiểm định trực tuyến
-2. Cổng tra cứu 12 điểm Giấy phép lái xe theo Luật mới 2026
-3. Hướng dẫn thủ tục sang tên xe theo Thông tư 24 &amp; danh bạ mã biển số 63 tỉnh thành
-Vai trò: Giải quyết nỗi lo pháp lý &amp; thu hút traffic SEO bền vững</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>Check-in Giữa Tháng 10 &amp; Review Cuối Tháng 10</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech &amp; VTTI | Content Team</t>
+      <c r="A13" s="85" t="n"/>
+      <c r="B13" s="87" t="inlineStr">
+        <is>
+          <t>Calculator</t>
+        </is>
+      </c>
+      <c r="C13" s="88" t="inlineStr">
+        <is>
+          <t>Công cụ Tài chính Xe (/lan-banh, /chi-phi-nuoi-xe, /so-sanh-xe)</t>
+        </is>
+      </c>
+      <c r="D13" s="88" t="inlineStr">
+        <is>
+          <t>Tính phí lăn bánh, chi phí nuôi xe, so sánh mẫu xe.</t>
+        </is>
+      </c>
+      <c r="E13" s="87" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
         </is>
       </c>
     </row>
     <row r="14" ht="68" customHeight="1">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Expansion &amp; Viral</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Phong Thủy &amp; Đấu Giá Biển Số (/bien-so-dep)</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>1. Công cụ giải mã ý nghĩa phong thủy 5 số cuối biển số xe (tính số nút, quẻ Dịch)
-2. Cập nhật kết quả đấu giá biển số đẹp định kỳ
-3. Động lực tự nhiên để người dùng tự nguyện nhập đủ biển số xe
-Vai trò: Viral Loop &amp; Khởi tạo Thẻ Xe Số (56.2K search)</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Giữa Tháng 10 &amp; Review Cuối Tháng 10</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech &amp; Content Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="68" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Phase 3: Scale-Up (Mở Rộng Quy Mô Dữ Liệu &amp; Hệ Sinh Thái - T11-12/2026)</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Vehicle Database (Scale-Up Dữ Liệu)</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Cơ Sở Dữ Liệu Hãng Xe &amp; Dòng Xe (/hang-xe/[brand]/[model])</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>1. Xây dựng trang cơ sở dữ liệu động cho toàn bộ thương hiệu xe (Toyota, Honda, VinFast, Ford, Mazda...)
-2. Sinh tự động hàng trăm trang chi tiết dòng xe (Specs, Bảng giá, Thư viện ảnh, Đánh giá ưu nhược điểm)
-3. Tích hợp Schema Car/Product chuẩn Google AIO
-Vai trò: Chiếm lĩnh toàn bộ từ khóa tên model xe trên Google</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>Check-in Sprint Tháng 11 &amp; Tháng 12</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech &amp; VTTI (Data)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="68" customHeight="1">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Mobility &amp; Smart City</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Trang Tra Cứu Bãi Đỗ Xe &amp; Camera Giao Thông Trên Web (/bai-do-xe, /camera-giao-thong)</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>• Xây dựng giao diện tra cứu bãi đỗ xe ô tô/xe máy VETC Parking tại Hà Nội &amp; TP.HCM trên Web.
-• Nhúng luồng live stream camera giao thông quan sát điểm kẹt xe, ngập nước thời gian thực.
-• Tích hợp bộ lọc bãi đỗ xe theo quận/huyện và nút chỉ đường Google Maps.</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Sprint Tháng 11 &amp; Tháng 12</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform | VTTI (Partner IoT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="68" customHeight="1">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Vehicle Profile &amp; In-App Sync</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Trang Hồ Sơ Phương Tiện &amp; Thu Thập Dữ Liệu Xe Trên Web (/ho-so-xe, /bao-hiem-o-to)</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>• Trang quản lý danh mục xe đã lưu trên Web và cổng liên kết tài khoản MoMo.
-• Thu thập dữ liệu biển số xe từ các phễu tra cứu Web để chuyển giao sang App.
-• Nút W2A dẫn người dùng vào màn hình mua Bảo hiểm In-App có sẵn Auto-fill (+10% CR).</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>Check-in Sprint Tháng 11 &amp; Tháng 12</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech Cell | VTTI (API)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="68" customHeight="1">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Partner Ecosystem</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Trang Danh Bạ &amp; Ưu Đãi Mạng Lưới Đối Tác Trên Web (/doi-tac, /doi-tac/[slug])</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>• Danh bạ thông tin các đối tác chiến lược (Petrolimex, VinFast, VETC, Bảo hiểm...).
-• Hiển thị chương trình ưu đãi độc quyền đối tác và nút nhận Voucher O2O.
-• Nâng tầm vị thế mặt tiền số 1 về tiện ích phương tiện tại Việt Nam.</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Check-in Sprint Tháng 11 &amp; Tháng 12</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform | InsurTech &amp; VTTI (Merchant)</t>
-        </is>
-      </c>
-    </row>
+      <c r="A14" s="86" t="n"/>
+      <c r="B14" s="87" t="inlineStr">
+        <is>
+          <t>Smart City</t>
+        </is>
+      </c>
+      <c r="C14" s="88" t="inlineStr">
+        <is>
+          <t>Camera &amp; Lộ trình (/camera-giao-thong, /chuyen-di)</t>
+        </is>
+      </c>
+      <c r="D14" s="88" t="inlineStr">
+        <is>
+          <t>Live stream camera điểm kẹt xe, nhật ký chuyến đi.</t>
+        </is>
+      </c>
+      <c r="E14" s="87" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="68" customHeight="1"/>
+    <row r="16" ht="68" customHeight="1"/>
+    <row r="17" ht="68" customHeight="1"/>
+    <row r="18" ht="68" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A4:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="A7:A9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1921,7 +1758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2181,122 +2018,122 @@
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>2. Pháp Lý, Vi Phạm &amp; Đăng Kiểm</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Thủ tục sang tên đổi chủ xe (/sang-ten-xe)</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>32000</v>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>0.2%</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>Informational / Legal</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Người mua/bán xe cũ tìm hiểu quy trình rút hồ sơ gốc và định danh biển số Thông tư 24.</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Cẩm nang pháp lý tạo uy tín thương hiệu; dẫn sang dịch vụ thanh toán thuế trước bạ.</t>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Tra cứu mức phạt giao thông NĐ 100/123 (/tra-cuu-vi-pham)</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Informational / Rule</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Người lái xe muốn tra cứu khung tiền phạt và thời hạn tước bằng lái khi phạm lỗi.</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Từ điển tra cứu nhanh; cảnh báo lỗi 'thiếu bảo hiểm' để bán chéo bảo hiểm TNDS 66k.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2. Pháp Lý, Vi Phạm &amp; Đăng Kiểm</t>
+          <t>3. Xe Điện &amp; Bảo Trì Phương Tiện</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Tra cứu mức phạt giao thông NĐ 100/123 (/tra-cuu-vi-pham)</t>
+          <t>Trạm sạc xe điện EV VinFast (/tram-sac)</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>25000</v>
+        <v>1240000</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Informational / Rule</t>
+          <t>Transactional / Local</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Người lái xe muốn tra cứu khung tiền phạt và thời hạn tước bằng lái khi phạm lỗi.</t>
+          <t>Chủ xe điện VinFast, V-Green tìm kiếm trụ sạc gần nhất dọc tuyến đường di chuyển.</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Từ điển tra cứu nhanh; cảnh báo lỗi 'thiếu bảo hiểm' để bán chéo bảo hiểm TNDS 66k.</t>
+          <t>Tiếp cận tệp khách hàng xe điện hiện đại (ARPU cao); bán chéo gói bảo hiểm xe điện.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="14" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2. Pháp Lý, Vi Phạm &amp; Đăng Kiểm</t>
+          <t>3. Xe Điện &amp; Bảo Trì Phương Tiện</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Tra cứu trừ điểm Giấy phép lái xe (/diem-gplx)</t>
+          <t>Sửa chữa &amp; Garage xe máy/ô tô (/tim-garage)</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>10000</v>
+        <v>934000</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Informational / Legal</t>
+          <t>Transactional / Emergency</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Tài xế theo dõi quy định trừ điểm bằng lái xe (12 điểm GPLX) theo Luật ATGT mới 2026.</t>
+          <t>Tài xế gặp sự cố hỏng hóc, thủng lốp hoặc cần tìm garage bảo dưỡng xe định kỳ uy tín.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Tiện ích đón đầu quy định mới; giữ chân tài xế và tăng độ phủ tìm kiếm AI Overview.</t>
+          <t>Bản đồ Garage Local GEO; dẫn dắt thanh toán dịch vụ sửa chữa qua Ví Trả Sau MoMo.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -2305,475 +2142,364 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Trạm sạc xe điện EV VinFast (/tram-sac)</t>
+          <t>Rửa xe &amp; Chăm sóc xe Detailing (/bao-duong)</t>
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1240000</v>
+        <v>284000</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>1.4%</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
+          <t>Commercial / Care</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Chủ xe tìm kiếm trung tâm detailing, rửa xe cao cấp, phủ ceramic hoặc dán phim cách nhiệt.</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Mạng lưới đối tác chăm sóc xe O2O; kết hợp phát hành voucher ưu đãi thành viên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>So sánh thông số mẫu xe (/so-sanh-xe)</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>0.2%</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Commercial / Research</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Khách hàng chuẩn bị mua xe cần đặt lên bàn cân đối chiếu 2-3 mẫu xe cùng tầm giá.</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Công cụ hỗ trợ quyết định mua xe; dẫn luồng sang tính giá lăn bánh và gói vay mua xe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Dự toán lệ phí trước bạ &amp; Giá lăn bánh (/lan-banh)</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>44000</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>0.2%</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>Commercial / Calc</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Người chuẩn bị mua xe mới/cũ muốn tính chính xác tổng chi phí thực tế phải nộp.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Máy tính dự toán lăn bánh 63 tỉnh; nguồn Lead chất lượng cho Bảo hiểm Ô tô &amp; Vay mua xe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Chi phí nuôi xe &amp; bảo trì hàng tháng (/chi-phi-nuoi-xe)</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>18500</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Informational / Finance</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Chủ xe tương lai muốn ước tính tổng chi phí xăng, gửi xe, bảo hiểm và bảo dưỡng.</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Công cụ lập ngân sách tài chính; kích hoạt tính năng Quản Lý Chi Tiêu trên MoMo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Định giá xe cũ &amp; Mua bán xe</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>14300</v>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Commercial / Value</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Chủ xe muốn định giá phương tiện đã qua sử dụng trước khi bán hoặc đổi xe mới.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Tiện ích định giá tham khảo; dẫn dắt luồng kết nối đối tác mua bán xe cũ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Bãi đỗ xe &amp; Giữ xe ô tô (/bai-do-xe)</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>180000</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>0.9%</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
           <t>Transactional / Local</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Chủ xe điện VinFast, V-Green tìm kiếm trụ sạc gần nhất dọc tuyến đường di chuyển.</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>Tiếp cận tệp khách hàng xe điện hiện đại (ARPU cao); bán chéo gói bảo hiểm xe điện.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>3. Xe Điện &amp; Bảo Trì Phương Tiện</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Sửa chữa &amp; Garage xe máy/ô tô (/tim-garage)</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>934000</v>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>4.6%</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>Transactional / Emergency</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Tài xế gặp sự cố hỏng hóc, thủng lốp hoặc cần tìm garage bảo dưỡng xe định kỳ uy tín.</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Bản đồ Garage Local GEO; dẫn dắt thanh toán dịch vụ sửa chữa qua Ví Trả Sau MoMo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>3. Xe Điện &amp; Bảo Trì Phương Tiện</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Rửa xe &amp; Chăm sóc xe Detailing (/bao-duong)</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>284000</v>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>1.4%</t>
-        </is>
-      </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>Commercial / Care</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Chủ xe tìm kiếm trung tâm detailing, rửa xe cao cấp, phủ ceramic hoặc dán phim cách nhiệt.</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>Mạng lưới đối tác chăm sóc xe O2O; kết hợp phát hành voucher ưu đãi thành viên.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Phong thủy &amp; Đấu giá biển số (/bien-so-dep)</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>56220</v>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>0.3%</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>Viral / Lifestyle</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Chủ xe vừa mua xe mới muốn xem ý nghĩa may mắn 5 số cuối và kết quả đấu giá biển đẹp.</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Đòn bẩy viral thu thập Biển số xe tự nguyện; dẫn sang tạo Thẻ Xe Số trên MoMo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>So sánh thông số mẫu xe (/so-sanh-xe)</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="n">
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Tài xế tìm kiếm bãi đỗ xe ô tô còn chỗ tại các khu vực trung tâm đông đúc.</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Bản đồ bãi đỗ VETC Parking; kích hoạt thanh toán trừ tiền tự động không cần dùng tiền mặt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Cứu hộ giao thông 24/7 khẩn cấp (/cuu-ho)</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>172000</v>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>0.9%</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Transactional / Urgent</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Tài xế gặp sự cố ngập nước, chết máy, nổ lốp cần gọi xe kéo cứu hộ khẩn cấp.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Hotline cứu hộ giao thông 24/7; liên kết đối tác cứu hộ uy tín toàn quốc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Biểu phí BOT &amp; Thu phí không dừng (/tram-thu-phi)</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>95000</v>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Commercial / Toll</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Tài xế chuẩn bị đi cao tốc muốn tra cứu mức phí trạm BOT và nạp tiền ePass/VETC.</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Dẫn luồng mở App MoMo nạp tiền thu phí không dừng và bật tính năng Auto-Topup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Camera giao thông quan sát kẹt xe (/camera)</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="n">
         <v>45000</v>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>0.2%</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>Commercial / Research</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Khách hàng chuẩn bị mua xe cần đặt lên bàn cân đối chiếu 2-3 mẫu xe cùng tầm giá.</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Công cụ hỗ trợ quyết định mua xe; dẫn luồng sang tính giá lăn bánh và gói vay mua xe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Dự toán lệ phí trước bạ &amp; Giá lăn bánh (/lan-banh)</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="n">
-        <v>44000</v>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>0.2%</t>
-        </is>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>Commercial / Calc</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Người chuẩn bị mua xe mới/cũ muốn tính chính xác tổng chi phí thực tế phải nộp.</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Máy tính dự toán lăn bánh 63 tỉnh; nguồn Lead chất lượng cho Bảo hiểm Ô tô &amp; Vay mua xe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Chi phí nuôi xe &amp; bảo trì hàng tháng (/chi-phi-nuoi-xe)</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>18500</v>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>0.1%</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>Informational / Finance</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Chủ xe tương lai muốn ước tính tổng chi phí xăng, gửi xe, bảo hiểm và bảo dưỡng.</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>Công cụ lập ngân sách tài chính; kích hoạt tính năng Quản Lý Chi Tiêu trên MoMo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>4. Mua Xe &amp; Dự Toán Chi Phí</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Định giá xe cũ &amp; Mua bán xe</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="n">
-        <v>14300</v>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>0.1%</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>Commercial / Value</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Chủ xe muốn định giá phương tiện đã qua sử dụng trước khi bán hoặc đổi xe mới.</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Tiện ích định giá tham khảo; dẫn dắt luồng kết nối đối tác mua bán xe cũ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="42" customHeight="1">
-      <c r="A21" s="12" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Bãi đỗ xe &amp; Giữ xe ô tô (/bai-do-xe)</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>180000</v>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>0.9%</t>
-        </is>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
-        <is>
-          <t>Transactional / Local</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>Tài xế tìm kiếm bãi đỗ xe ô tô còn chỗ tại các khu vực trung tâm đông đúc.</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Bản đồ bãi đỗ VETC Parking; kích hoạt thanh toán trừ tiền tự động không cần dùng tiền mặt.</t>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Informational / Live</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Người đi đường muốn xem hình ảnh camera trực tiếp tránh các điểm ùn tắc, ngập lụt.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Tiện ích giữ chân người dùng trong giờ cao điểm; khẳng định vị thế Super App.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Cứu hộ giao thông 24/7 khẩn cấp (/cuu-ho)</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="n">
-        <v>172000</v>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>0.9%</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>Transactional / Urgent</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Tài xế gặp sự cố ngập nước, chết máy, nổ lốp cần gọi xe kéo cứu hộ khẩn cấp.</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Hotline cứu hộ giao thông 24/7; liên kết đối tác cứu hộ uy tín toàn quốc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="12" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Biểu phí BOT &amp; Thu phí không dừng (/tram-thu-phi)</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="n">
-        <v>95000</v>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>0.5%</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>Commercial / Toll</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Tài xế chuẩn bị đi cao tốc muốn tra cứu mức phí trạm BOT và nạp tiền ePass/VETC.</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>Dẫn luồng mở App MoMo nạp tiền thu phí không dừng và bật tính năng Auto-Topup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>5. Di Chuyển &amp; Hạ Tầng Đô Thị</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Camera giao thông quan sát kẹt xe (/camera)</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>45000</v>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>0.2%</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>Informational / Live</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Người đi đường muốn xem hình ảnh camera trực tiếp tránh các điểm ùn tắc, ngập lụt.</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Tiện ích giữ chân người dùng trong giờ cao điểm; khẳng định vị thế Super App.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="62" t="inlineStr"/>
-      <c r="B25" s="76" t="inlineStr">
+      <c r="A22" s="62" t="inlineStr"/>
+      <c r="B22" s="76" t="inlineStr">
         <is>
           <t>TỔNG CỘNG QUY MÔ TOÀN BỘ THỊ TRƯỜNG</t>
         </is>
       </c>
-      <c r="C25" s="76" t="inlineStr">
+      <c r="C22" s="76" t="inlineStr">
         <is>
           <t>20 Chủ Đề Nhu Cầu Tiện Ích Giao Thông</t>
         </is>
       </c>
-      <c r="D25" s="77" t="n">
+      <c r="D22" s="77" t="n">
         <v>20106020</v>
       </c>
-      <c r="E25" s="62" t="inlineStr">
+      <c r="E22" s="62" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="F25" s="76" t="inlineStr"/>
-      <c r="G25" s="76" t="inlineStr"/>
-      <c r="H25" s="76" t="inlineStr"/>
-    </row>
+      <c r="F22" s="76" t="inlineStr"/>
+      <c r="G22" s="76" t="inlineStr"/>
+      <c r="H22" s="76" t="inlineStr"/>
+    </row>
+    <row r="23" ht="42" customHeight="1"/>
+    <row r="24" ht="42" customHeight="1"/>
+    <row r="25" ht="26" customHeight="1"/>
     <row r="26" ht="30" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2781,6 +2507,252 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="101" t="inlineStr">
+        <is>
+          <t>Nhóm Tính Năng</t>
+        </is>
+      </c>
+      <c r="B1" s="101" t="inlineStr">
+        <is>
+          <t>Tên Trang (URL)</t>
+        </is>
+      </c>
+      <c r="C1" s="101" t="inlineStr">
+        <is>
+          <t>Content Structure (Trình tự Block từ trên xuống)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>Master Hub</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>Trang Chủ
+(/tien-ich-giao-thong)</t>
+        </is>
+      </c>
+      <c r="C2" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Component tra cứu
+2. Metric
+3. Giá Xăng + Cây Xăng
+4. Garage
+5. Cross-Sell Bảo Hiểm Ô tô/xe máy
+6. FAQ
+7. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="81" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="B3" s="81" t="inlineStr">
+        <is>
+          <t>Cổng Tra Cứu Phạt Nguội
+(/phat-nguoi)</t>
+        </is>
+      </c>
+      <c r="C3" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Search Box nhập biển số
+2. Result Component (Trả kết quả Lỗi / Không lỗi)
+3. Cross-Sell Bảo Hiểm &amp; CTA Nộp phạt In-App
+4. Bảng tra cứu mã lỗi phổ biến (NĐ 100/123)
+5. Cụm liên kết Location Page (Phạt nguội theo Tỉnh/Thành)
+6. FAQ
+7. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="81" t="inlineStr">
+        <is>
+          <t>Location &amp; Maps</t>
+        </is>
+      </c>
+      <c r="B4" s="81" t="inlineStr">
+        <is>
+          <t>Giá Xăng &amp; Cây Xăng
+(/gia-xang, /cay-xang)</t>
+        </is>
+      </c>
+      <c r="C4" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Bảng Giá xăng cập nhật Realtime
+2. Component Bản đồ (Định vị GPS Cây xăng gần nhất)
+3. Metric (Lịch sử biến động giá)
+4. Component Calculator (Tính tiền đầy bình)
+5. Cross-Sell (Bảo hiểm hoặc CTA Mở App)
+6. FAQ
+7. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="81" t="inlineStr">
+        <is>
+          <t>Location &amp; Maps</t>
+        </is>
+      </c>
+      <c r="B5" s="81" t="inlineStr">
+        <is>
+          <t>Trạm Sạc Xe Điện EV
+(/tram-sac)</t>
+        </is>
+      </c>
+      <c r="C5" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Search Box khu vực
+2. Component Bản đồ (Định vị Trạm sạc VinFast/V-Green)
+3. Filter Component (Lọc trạm AC/DC)
+4. Cross-Sell Bảo Hiểm Ô tô
+5. FAQ
+6. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="81" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B6" s="81" t="inlineStr">
+        <is>
+          <t>Tra Cứu Hạn Đăng Kiểm
+(/dang-kiem)</t>
+        </is>
+      </c>
+      <c r="C6" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Component Tra cứu Hạn Đăng kiểm
+2. Kết quả chu kỳ &amp; Countdown ngày hết hạn
+3. Component Đặt lịch kiểm định
+4. Cross-Sell Bảo Hiểm (Bắt buộc mang theo khi kiểm định)
+5. Bảng chu kỳ kiểm định các loại xe
+6. FAQ
+7. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="81" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="B7" s="81" t="inlineStr">
+        <is>
+          <t>Thu Phí Không Dừng
+(/phi-khong-dung)</t>
+        </is>
+      </c>
+      <c r="C7" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Component Tra cứu tài khoản ePass/VETC
+2. CTA Liên kết &amp; Nạp tiền tự động
+3. Bảng cước phí trạm thu phí BOT
+4. Hướng dẫn dán thẻ
+5. FAQ
+6. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="81" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="B8" s="81" t="inlineStr">
+        <is>
+          <t>Cứu Hộ Ô Tô
+(/cuu-ho)</t>
+        </is>
+      </c>
+      <c r="C8" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Dropdown chọn Vị trí
+2. Component Bản đồ &amp; Danh sách Garage Cứu hộ 24/7
+3. Hotline Component (SOS Click-to-call)
+4. Bảng giá dịch vụ khẩn cấp tham khảo
+5. FAQ
+6. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>Monetize</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="inlineStr">
+        <is>
+          <t>Bảo Hiểm Phương Tiện
+(/bao-hiem-o-to)</t>
+        </is>
+      </c>
+      <c r="C9" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Bảng so sánh 9 hãng bảo hiểm
+2. Component Nhập thông tin xe (Auto-fill)
+3. Bảng quyền lợi &amp; CTA Mua ngay
+4. Metric (Lượt bồi thường, uy tín)
+5. FAQ
+6. Long Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="81" t="inlineStr">
+        <is>
+          <t>Calculator</t>
+        </is>
+      </c>
+      <c r="B10" s="81" t="inlineStr">
+        <is>
+          <t>Công cụ Chi phí Lăn Bánh
+(/lan-banh)</t>
+        </is>
+      </c>
+      <c r="C10" s="102" t="inlineStr">
+        <is>
+          <t>1. Hero Section: H1 + Form chọn Hãng/Dòng xe/Tỉnh thành
+2. Component Bảng tính chi phí lăn bánh chi tiết
+3. Cross-Sell (Bảo hiểm xe mới / Vay mua xe)
+4. FAQ
+5. Long Content</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2998,7 +2970,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3744,13 +3716,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4035,81 +4007,32 @@
       </c>
     </row>
     <row r="9" ht="80" customHeight="1">
-      <c r="A9" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Giải Mã Phong Thủy &amp; Quẻ Dịch Biển Số Xe</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Viral Mini-App / Interactive Result Card</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Giải mã ý nghĩa may mắn, tính số nút và tra cứu quẻ phong thủy 5 số cuối của biển số xe.</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>• 5 chữ số cuối của biển số xe (VD: 12345)</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>1. Tính Số Nút (1-10): Nut = (d1 + d2 + d3 + d4 + d5) mod 10 (Nếu = 0 là 10 nút).
-2. Quẻ Phong Thủy 80 Linh Số: Index = ((5_digits / 80) - INT(5_digits / 80)) * 80. Lấy phần nguyên tra cứu 80 quẻ cát/hung.
-3. Nhận diện cặp số phong thủy: Thần tài (39, 79), Lộc phát (68, 86), Ông địa (38, 78), Tứ quý, Ngũ quý.</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>• Điểm phong thủy biển số (Thang điểm 10).
-• Lời bình quẻ dịch (Đại Cát, Cát, Bình An, Hung).
-• Ý nghĩa số nút và cặp số tài lộc.</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>Nút 'Lưu Biển Số Hợp Mệnh Vào Ví MoMo' để kích hoạt Thẻ Xe Số cá nhân.</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>Nhúng linh hoạt: Trang Đấu giá biển số, Trang Tra cứu phạt nguội, Trang chủ Hub, Social Sharing Card, In-App Minigame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="80" customHeight="1">
-      <c r="A10" s="14" t="n">
+      <c r="A9" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Tra Cứu Chu Kỳ &amp; Hạn Đăng Kiểm Tự Động</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Timeline Widget / Alert Card</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Tra cứu chu kỳ kiểm định và tính chính xác ngày hết hạn đăng kiểm để không bị phạt tiền quá hạn.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>• Loại phương tiện (Ô tô con không KD, Có KD, Ô tô tải)
 • Năm sản xuất xe (Year_prod)
 • Ngày đăng kiểm gần nhất (Date_last)</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>1. Tuổi xe: Age = Current_Year - Year_prod.
 2. Xác định chu kỳ kiểm định (Thông tư 02/2023/TT-BGTVT): Xe con không KD: Đến 7 năm = 24 tháng; Từ 7-20 năm = 12 tháng; Trên 20 năm = 6 tháng.
@@ -4117,100 +4040,48 @@
 4. Số ngày còn lại: Days_Left = Date_expiry - Current_Date.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>• Ngày hết hạn đăng kiểm chính xác.
 • Trạng thái hạn kiểm định (Còn hạn / Sắp hết hạn &lt;30 ngày / Quá hạn vi phạm).</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Nút 'Bật Nhắc Hạn Đăng Kiểm Tự Động' qua thông báo Notification App MoMo.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Nhúng linh hoạt: Trang Đăng kiểm xe, Sổ Garage số, Trang Phạt nguội, Trang Bảo hiểm ô tô, Email/ZNS nhắc hạn.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Từ Điển Tra Cứu Mức Phạt &amp; 12 Điểm GPLX</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Instant Search Filter / Table Drawer</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Tra cứu nhanh khung tiền phạt, thời gian tước bằng lái và số điểm GPLX bị trừ theo luật mới.</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>• Loại phương tiện (Ô tô, Xe máy)
-• Từ khóa hành vi vi phạm (Nồng độ cồn, Tốc độ, Đèn đỏ, Thiếu bảo hiểm...)</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Query Căn cứ Nghị định 100/2019/NĐ-CP, NĐ 123/2021/NĐ-CP &amp; Luật Trật tự ATGT đường bộ 2024:
-1. Khung tiền phạt: Min_Fine, Max_Fine, Avg_Fine.
-2. Tước quyền sử dụng GPLX: 0 - 24 tháng.
-3. Trừ điểm bằng lái xe: 0 - 12 điểm GPLX.
-4. Tạm giữ phương tiện: Có/Không (theo quy định).</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>• Khung tiền phạt chi tiết (VD: 4.000.000đ - 6.000.000đ).
-• Số điểm GPLX bị trừ (VD: Bị trừ 3 điểm).
-• Trích dẫn điều khoản luật chính xác.</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Nút 'Mua Bảo Hiểm TNDS Bắt Buộc 66K' (để tránh lỗi phạt 100k-200k khi CSGT kiểm tra).</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Nhúng linh hoạt: Trang Tra cứu vi phạm, Trang Phạt nguội, Trang Điểm GPLX, Các bài viết cẩm nang luật giao thông.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="14" t="n">
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Công Cụ Đặt Lên Bàn Cân So Sánh Xe</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Side-by-Side Comparison Matrix / Floating Comparison Bar</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Đặt lên bàn cân đối chiếu trực quan 30+ thông số kỹ thuật và trang bị giữa 2-3 mẫu xe cùng tầm giá.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>• Chọn Mẫu Xe A vs Mẫu Xe B (vs Mẫu Xe C)</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Thuật toán đối chiếu Side-by-Side 30+ trường dữ liệu:
 1. Kích thước (D x R x C, Trục cơ sở, Khoảng sáng gầm).
@@ -4220,30 +4091,32 @@
 =&gt; Tự động Highlight thông số vượt trội (Xanh lá).</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>• Bảng đối chiếu Side-by-Side toàn diện.
 • Đánh giá ưu điểm / nhược điểm của từng mẫu xe.
 • Điểm chấm tổng quan (MoMo Vehicle Rating).</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Nút 'Tính Chi Phí Lăn Bánh Chi Tiết' &amp; 'Đăng Ký Lái Thử / Nhận Ưu Đãi'.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Nhúng linh hoạt: Trang So sánh xe, Trang Danh mục Hãng xe, Trang chi tiết Dòng xe, Bài viết review phân khúc xe.</t>
         </is>
       </c>
     </row>
+    <row r="11" ht="80" customHeight="1"/>
+    <row r="12" ht="80" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>